<commit_message>
feat: Guest booking wizard, admin approval flow, guest account management
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,10 +768,8 @@
           <t>d</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1234567891</t>
-        </is>
+      <c r="D9" t="n">
+        <v>1234567891</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
@@ -793,6 +791,46 @@
       <c r="J9" t="inlineStr">
         <is>
           <t>2026-03-21T02:33:40.942706</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>concakpvp</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0364216007</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>concakpvp123@gmail.com</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:50:11.587830</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:50:11.587830</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fix My Room data binding, admin notifications for repairs with persistence, admin logout, guest routing fix
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -806,10 +806,8 @@
           <t>concakpvp</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>0364216007</t>
-        </is>
+      <c r="D10" t="n">
+        <v>364216007</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -831,6 +829,100 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>2026-03-21T04:50:11.587830</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Guest Test 22</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Test address</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-03-21T05:57:24.583588</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-03-21T05:57:24.583588</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Guest Test 22</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Test address</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-03-21T05:57:49.585286</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-03-21T05:57:49.585286</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix guest personal info, add validation, auto-fill booking, and fix admin bank info UI/persistence
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,16 @@
           <t>updated_at</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dob</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -511,6 +521,8 @@
           <t>2025-01-01</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -555,6 +567,8 @@
           <t>2025-01-01</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -599,6 +613,8 @@
           <t>2025-01-10</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -643,6 +659,8 @@
           <t>2025-01-01</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -687,6 +705,8 @@
           <t>2024-06-01</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -725,6 +745,8 @@
           <t>2026-03-21T02:09:01.539450</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -755,6 +777,8 @@
           <t>2026-03-21T02:21:57.964195</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -793,6 +817,8 @@
           <t>2026-03-21T02:33:40.942706</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -816,7 +842,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>012345678901</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -828,7 +854,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:50:11.587830</t>
+          <t>2026-03-21T17:08:40.031638</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>13/7/2008</t>
         </is>
       </c>
     </row>
@@ -877,6 +913,8 @@
           <t>2026-03-21T05:57:24.583588</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -890,16 +928,14 @@
           <t>Guest Test 22</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>123456789012</t>
@@ -923,6 +959,58 @@
       <c r="J12" t="inlineStr">
         <is>
           <t>2026-03-21T05:57:49.585286</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1111111111</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>11@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>123456789112</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-21T16:54:01.246614</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-03-21T17:50:53.717301</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>7/8/2003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guest: notification/avatar dropdowns, logout confirmation, priority combobox, fix crashes
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -976,10 +976,8 @@
           <t>Test User</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1111111111</t>
-        </is>
+      <c r="D13" t="n">
+        <v>1111111111</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1011,6 +1009,104 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>7/8/2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Quỳnh My</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>869223246</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>quynhmyy987@gmail.com</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>111111111111</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-21T20:21:29.607042</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-03-21T20:21:35.671055</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0333333333</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>33@gmail.com</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-21T20:45:05.953133</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-03-21T20:45:05.953133</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>7/9/2003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Cập nhật dữ liệu và thêm debug script - Cập nhật data: guests, invoices, rooms, users, contracts, notifications - Thêm room images P204 - Thêm debug_dashboard.py
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1072,10 +1072,8 @@
           <t>33</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0333333333</t>
-        </is>
+      <c r="D15" t="n">
+        <v>333333333</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1107,6 +1105,56 @@
       <c r="L15" t="inlineStr">
         <is>
           <t>7/9/2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Khoa Trịnh</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>khoattd22411@gmail.com</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-22T04:03:00.666879</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-03-22T04:03:10.719243</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>8/7/2002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: Thêm Matplotlib/Seaborn/Numpy vào dashboard, cập nhật thông tin chủ trọ, xóa file debug
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1120,10 +1120,8 @@
           <t>Khoa Trịnh</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>123456789</t>
-        </is>
+      <c r="D16" t="n">
+        <v>123456789</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1155,6 +1153,152 @@
       <c r="L16" t="inlineStr">
         <is>
           <t>8/7/2002</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>123423456</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>khanhkhanh190727@gmail.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-24T22:55:45.623840</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-03-24T22:55:51.254584</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" t="n">
+        <v>11</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Đan ngu ăn cứt chó</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>345787652</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>lethedan0707@gmail.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-24T23:37:14.362605</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-03-24T23:37:21.166814</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Guest 44</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>123141234222</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-25T01:20:04.554753</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-03-25T01:20:04.554753</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: thêm đổi phòng, cài đặt hệ thống, sửa dropdown repair + xóa session_timeout
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>concakpvp123@gmail.com</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-03-25T01:20:04.554753</t>
+          <t>2026-03-27T00:39:43.810728</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">

</xml_diff>

<commit_message>
Fix CCCD data type, update invoice service, and UI improvements
</commit_message>
<xml_diff>
--- a/Ma_Nguon/data/excel/guests.xlsx
+++ b/Ma_Nguon/data/excel/guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,16 +490,20 @@
           <t>concakpvp</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>364216007</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0364216007</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>concakpvp123@gmail.com</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>123456789012</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -510,7 +514,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-27T15:04:06.442421</t>
+          <t>2026-04-01T04:23:53.293735</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -518,41 +522,49 @@
           <t>Nam</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>2007</v>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>4/7/2002</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>concakpvp</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>364216007</v>
+          <t>Toàn Lê</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>123456765</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>concakpvp123@gmail.com</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>ngoctoanle266@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-27T15:04:13.269184</t>
+          <t>2026-03-27T15:21:51.642782</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-03-27T15:04:13.269184</t>
+          <t>2026-04-01T02:53:15.461800</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -562,57 +574,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>8/7/2003</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Toàn Lê</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>123456765</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ngoctoanle266@gmail.com</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>012345678912</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-03-27T15:21:51.642782</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2026-03-27T15:22:01.177009</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Nam</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2007</t>
+          <t>6/5/2007</t>
         </is>
       </c>
     </row>

</xml_diff>